<commit_message>
Integrate Sustainary funding monitor
</commit_message>
<xml_diff>
--- a/outputs/dansk_fonds_database.xlsx
+++ b/outputs/dansk_fonds_database.xlsx
@@ -2,8 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonde" sheetId="1" r:id="R81cc2e450ed74372"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opsummering" sheetId="2" r:id="Re257d46f10d14aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonde" sheetId="1" r:id="R8ce1197ec5b543df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puljer" sheetId="2" r:id="R2bef05ec2eba43e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frister" sheetId="3" r:id="Rd794346f787f46f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opsummering" sheetId="4" r:id="R2412d0086b9947af"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -86,9 +88,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -101,12 +103,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -241,10 +289,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>novo-nordisk-fonden</x:v>
+        <x:v>nordea-fonden</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Novo Nordisk Fonden</x:v>
+        <x:v>Nordea-fonden</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -256,75 +304,75 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Hellerup</x:v>
+        <x:v>København</x:v>
       </x:c>
       <x:c r="G2" t="str">
-        <x:v>https://novonordiskfonden.dk</x:v>
+        <x:v>https://nordeafonden.dk</x:v>
       </x:c>
       <x:c r="H2" t="str">
-        <x:v>https://novonordiskfonden.dk/en/apply-for-grants/</x:v>
+        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="I2" t="str">
-        <x:v>Sundhed; biovidenskab; naturvidenskab; teknologi; uddannelse; kunsthistorisk forskning; samfundsmæssig bæredygtighed</x:v>
+        <x:v>Sundhed; motion; natur; kultur; fællesskaber; gode liv</x:v>
       </x:c>
       <x:c r="J2" t="str">
-        <x:v>Forskningsinstitutioner; organisationer; projekter efter opslag</x:v>
+        <x:v>Foreninger; organisationer; institutioner; lokale projekter</x:v>
       </x:c>
       <x:c r="K2" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Løbende og puljer</x:v>
       </x:c>
       <x:c r="L2" t="str">
-        <x:v>Ansøgninger indsendes typisk via NORMA og afhænger af konkrete calls.</x:v>
+        <x:v>Filantropisk fond med fokus på gode liv i Danmark.</x:v>
       </x:c>
       <x:c r="M2" t="str">
-        <x:v>https://novonordiskfonden.dk/en/how-we-work/what-are-grants/applying-for-a-grant/</x:v>
+        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="N2" t="str">
         <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="O2" t="str">
-        <x:v>source_checked</x:v>
+        <x:v>to_verify</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>realdania</x:v>
+        <x:v>trygfonden</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Realdania</x:v>
+        <x:v>TrygFonden</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Forening/fondslignende filantropisk aktør</x:v>
+        <x:v>Almennyttig fond/fondslignende</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>Ikke relevant/forening</x:v>
+        <x:v>To verify</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>København</x:v>
+        <x:v>Kgs. Lyngby</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>https://realdania.dk</x:v>
+        <x:v>https://tryghed.dk</x:v>
       </x:c>
       <x:c r="H3" t="str">
-        <x:v>https://realdania.dk/soeg-stoette</x:v>
+        <x:v>https://tryghed.dk/sog-stotte</x:v>
       </x:c>
       <x:c r="I3" t="str">
-        <x:v>Bygninger; byer; byrum; bygningsarv; fællesskaber; livskvalitet</x:v>
+        <x:v>Tryghed; sundhed; sikkerhed; trivsel; forskning; beredskab</x:v>
       </x:c>
       <x:c r="J3" t="str">
-        <x:v>Organisationer; kommuner; foreninger; professionelle projektaktører</x:v>
+        <x:v>Organisationer; institutioner; NGO'er; frivillige; forskere</x:v>
       </x:c>
       <x:c r="K3" t="str">
-        <x:v>Løbende og tematiske indsatser</x:v>
+        <x:v>Løbende og landsdækkende puljer</x:v>
       </x:c>
       <x:c r="L3" t="str">
-        <x:v>Støtter projekter med tilknytning til det byggede miljø.</x:v>
+        <x:v>Støtter ikke privatpersoner og ikke kommercielle, politiske eller religiøse projekter.</x:v>
       </x:c>
       <x:c r="M3" t="str">
-        <x:v>https://realdania.dk/soeg-stoette</x:v>
+        <x:v>https://tryghed.dk/sog-stotte</x:v>
       </x:c>
       <x:c r="N3" t="str">
         <x:v>2026-06-08</x:v>
@@ -335,10 +383,10 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>nordea-fonden</x:v>
+        <x:v>villum-fonden</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Nordea-fonden</x:v>
+        <x:v>VILLUM FONDEN</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -350,42 +398,42 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>København</x:v>
+        <x:v>Søborg</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>https://nordeafonden.dk</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
       </x:c>
       <x:c r="I4" t="str">
-        <x:v>Sundhed; motion; natur; kultur; fællesskaber; gode liv</x:v>
+        <x:v>Teknisk og naturvidenskabelig forskning; miljø og klima; børn unge og science; unge og uddannelse; kultur og samfund</x:v>
       </x:c>
       <x:c r="J4" t="str">
-        <x:v>Foreninger; organisationer; institutioner; lokale projekter</x:v>
+        <x:v>Forskere; institutioner; organisationer; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K4" t="str">
-        <x:v>Løbende og puljer</x:v>
+        <x:v>Opslag/calls</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>Filantropisk fond med fokus på gode liv i Danmark.</x:v>
+        <x:v>Relevant ved opslag om unge, uddannelse, miljø og klima.</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O4" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>trygfonden</x:v>
+        <x:v>velux-fonden</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>TrygFonden</x:v>
+        <x:v>VELUX FONDEN</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>Almennyttig fond/fondslignende</x:v>
@@ -397,31 +445,31 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Kgs. Lyngby</x:v>
+        <x:v>Søborg</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>https://tryghed.dk</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>https://tryghed.dk/sog-stotte</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
       </x:c>
       <x:c r="I5" t="str">
-        <x:v>Tryghed; sundhed; sikkerhed; trivsel; forskning; beredskab</x:v>
+        <x:v>Demokratisk bæredygtighed; sociale indsatser; human- og samfundsvidenskab; havmiljø</x:v>
       </x:c>
       <x:c r="J5" t="str">
-        <x:v>Organisationer; institutioner; NGO'er; frivillige; forskere</x:v>
+        <x:v>Forskere; praktikere; institutioner; organisationer; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K5" t="str">
-        <x:v>Løbende og landsdækkende puljer</x:v>
+        <x:v>Opslag/calls</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>Støtter ikke privatpersoner og ikke kommercielle, politiske eller religiøse projekter.</x:v>
+        <x:v>Stærkt match ved opslag om demokratisk bæredygtighed og sociale indsatser.</x:v>
       </x:c>
       <x:c r="M5" t="str">
-        <x:v>https://tryghed.dk/sog-stotte</x:v>
+        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O5" t="str">
         <x:v>source_checked</x:v>
@@ -429,10 +477,10 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>villum-fonden</x:v>
+        <x:v>bikubenfonden</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>VILLUM FONDEN</x:v>
+        <x:v>Bikubenfonden</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -444,28 +492,28 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Søborg</x:v>
+        <x:v>København</x:v>
       </x:c>
       <x:c r="G6" t="str">
-        <x:v>https://veluxfoundations.dk</x:v>
+        <x:v>https://www.bikubenfonden.dk</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>https://veluxfoundations.dk/en/apply-grant/villum-fonden</x:v>
+        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="I6" t="str">
-        <x:v>Teknisk og naturvidenskabelig forskning; miljø; børn og unge; sociale indsatser</x:v>
+        <x:v>Billedkunst; scenekunst; unge på kanten; sociale forandringer</x:v>
       </x:c>
       <x:c r="J6" t="str">
-        <x:v>Forskere; institutioner; organisationer; projekter efter opslag</x:v>
+        <x:v>Kunstnere; kulturinstitutioner; sociale organisationer; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K6" t="str">
         <x:v>Opslag/calls</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>En del af THE VELUX FOUNDATIONS.</x:v>
+        <x:v>Fokus på kunst og sociale indsatser.</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>https://veluxfoundations.dk/en/apply-grant/villum-fonden</x:v>
+        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="N6" t="str">
         <x:v>2026-06-08</x:v>
@@ -476,10 +524,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>velux-fonden</x:v>
+        <x:v>tuborgfondet</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>VELUX FONDEN</x:v>
+        <x:v>Tuborgfondet</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>Almennyttig fond/fondslignende</x:v>
@@ -491,28 +539,28 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Søborg</x:v>
+        <x:v>København</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>https://veluxfoundations.dk</x:v>
+        <x:v>https://www.tuborgfondet.dk</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>https://veluxfoundations.dk/en/apply-grant/velux-fonden</x:v>
+        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
       </x:c>
       <x:c r="I7" t="str">
-        <x:v>Aldrende samfund; humanvidenskab; demokrati; bæredygtighed; øjenforskning; sociale indsatser</x:v>
+        <x:v>Unge; fællesskaber; demokrati; grøn omstilling; civilsamfund</x:v>
       </x:c>
       <x:c r="J7" t="str">
-        <x:v>Forskere; institutioner; organisationer; projekter efter opslag</x:v>
+        <x:v>Unge; foreninger; organisationer; lokale initiativer</x:v>
       </x:c>
       <x:c r="K7" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Løbende og puljer</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>En del af THE VELUX FOUNDATIONS.</x:v>
+        <x:v>Fokus på unges engagement og handlekraft.</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>https://veluxfoundations.dk/en/apply-grant/velux-fonden</x:v>
+        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
       </x:c>
       <x:c r="N7" t="str">
         <x:v>2026-06-08</x:v>
@@ -523,10 +571,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>lundbeckfonden</x:v>
+        <x:v>egmont-fonden</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>Lundbeckfonden</x:v>
+        <x:v>Egmont Fonden</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -541,25 +589,25 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>https://lundbeckfonden.com</x:v>
+        <x:v>https://www.egmontfonden.dk</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>https://lundbeckfonden.com/grants/</x:v>
+        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
       </x:c>
       <x:c r="I8" t="str">
-        <x:v>Biomedicin; sundhedsvidenskab; neuroscience; forskning; talentudvikling</x:v>
+        <x:v>Børn og unge; udsathed; læring; trivsel; social mobilitet</x:v>
       </x:c>
       <x:c r="J8" t="str">
-        <x:v>Forskere; forskningsinstitutioner; startups efter program</x:v>
+        <x:v>Organisationer; institutioner; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K8" t="str">
         <x:v>Opslag/calls</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>Fokus på biomedicinsk forskning og bedre hjernesundhed.</x:v>
+        <x:v>Fokus på børn og unge i udsatte positioner.</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>https://lundbeckfonden.com/grants/</x:v>
+        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
       </x:c>
       <x:c r="N8" t="str">
         <x:v>2026-06-08</x:v>
@@ -570,10 +618,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>carlsbergfondet</x:v>
+        <x:v>lauritzen-fonden</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>Carlsbergfondet</x:v>
+        <x:v>Lauritzen Fonden</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -585,89 +633,89 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>København</x:v>
+        <x:v>Hellerup</x:v>
       </x:c>
       <x:c r="G9" t="str">
-        <x:v>https://carlsbergfondet.dk</x:v>
+        <x:v>https://lauritzenfonden.com</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>https://carlsbergfondet.dk/ansoeger/</x:v>
+        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
       </x:c>
       <x:c r="I9" t="str">
-        <x:v>Fri grundforskning; naturvidenskab; samfundsvidenskab; humaniora; forskningsinfrastruktur; formidling</x:v>
+        <x:v>Udsatte børn og unge; maritimt; uddannelse; kultur; humanitære indsatser</x:v>
       </x:c>
       <x:c r="J9" t="str">
-        <x:v>Forskere med dansk forskningsmiljø-tilknytning; institutioner</x:v>
+        <x:v>Organisationer; institutioner; projekter</x:v>
       </x:c>
       <x:c r="K9" t="str">
-        <x:v>Årlige opslag/calls</x:v>
+        <x:v>Løbende og opslag</x:v>
       </x:c>
       <x:c r="L9" t="str">
-        <x:v>Støtter fri grundforskning i åben konkurrence.</x:v>
+        <x:v>Har historisk maritime rødder og bred almennyttig uddeling.</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>https://carlsbergfondet.dk/bevillingsenhed/vores-forskningsstoette/</x:v>
+        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
       </x:c>
       <x:c r="N9" t="str">
         <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>source_checked</x:v>
+        <x:v>to_verify</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>ap-moeller-fonden</x:v>
+        <x:v>ole-kirks-fond</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>A.P. Møller Fonden</x:v>
+        <x:v>Ole Kirk's Fond</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>Erhvervsdrivende fond</x:v>
+        <x:v>Almennyttig fond/fondslignende</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Erhvervsstyrelsen</x:v>
+        <x:v>To verify</x:v>
       </x:c>
       <x:c r="E10" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>København</x:v>
+        <x:v>Billund</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>https://www.apmollerfonde.dk</x:v>
+        <x:v>https://olekirksfond.dk</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>https://www.apmollerfonde.dk/ansoegning/a-p-moeller-fonden/</x:v>
+        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
       </x:c>
       <x:c r="I10" t="str">
-        <x:v>Almennyttige formål; Norden; dansk-tyske grænseland; dansk søfart og industri; videnskab; lægevidenskab</x:v>
+        <x:v>Børn; familier; trivsel; leg; læring; sociale indsatser</x:v>
       </x:c>
       <x:c r="J10" t="str">
-        <x:v>Organisationer; institutioner; projekter med CVR</x:v>
+        <x:v>Organisationer; institutioner; projekter</x:v>
       </x:c>
       <x:c r="K10" t="str">
-        <x:v>Løbende</x:v>
+        <x:v>Løbende og opslag</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>Behandler ikke ansøgninger sendt pr. e-mail; ansøgning via portal.</x:v>
+        <x:v>Fokus på børns og familiers muligheder.</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>https://www.apmollerfonde.dk/ansoegning/a-p-moeller-fonden/</x:v>
+        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
       </x:c>
       <x:c r="N10" t="str">
         <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>source_checked</x:v>
+        <x:v>to_verify</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>augustinus-fonden</x:v>
+        <x:v>kr-foundation</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>Augustinus Fonden</x:v>
+        <x:v>KR Foundation</x:v>
       </x:c>
       <x:c r="C11" t="str">
         <x:v>Almennyttig fond/fondslignende</x:v>
@@ -682,45 +730,45 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>https://augustinusfonden.dk</x:v>
+        <x:v>https://krfnd.org</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>https://augustinusfonden.dk/da/sadan-kommer-du-i-gang</x:v>
+        <x:v>https://krfnd.org/apply-for-funding/</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>Kunst; kultur; kulturarv; sociale indsatser; vidensprojekter</x:v>
+        <x:v>Klima; bæredygtighed; systemforandring; adfærd; policy</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>Organisationer; institutioner; professionelle aktører</x:v>
+        <x:v>Organisationer; NGO'er; internationale partnerskaber</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>Afhænger af støtteområde</x:v>
+        <x:v>Opslag/invitation</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>Krav, kriterier og frister varierer efter støtteområde.</x:v>
+        <x:v>International klimafond med dansk base.</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>https://augustinusfonden.dk/da/sadan-kommer-du-i-gang</x:v>
+        <x:v>https://krfnd.org/apply-for-funding/</x:v>
       </x:c>
       <x:c r="N11" t="str">
         <x:v>2026-06-08</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>source_checked</x:v>
+        <x:v>to_verify</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>bikubenfonden</x:v>
+        <x:v>duf</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>Bikubenfonden</x:v>
+        <x:v>Dansk Ungdoms Fællesråd (DUF)</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>Erhvervsdrivende fond</x:v>
+        <x:v>Paraplyorganisation/fondslignende puljeaktør</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>Erhvervsstyrelsen</x:v>
+        <x:v>Ikke relevant/forening</x:v>
       </x:c>
       <x:c r="E12" t="str">
         <x:v>Danmark</x:v>
@@ -729,92 +777,90 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G12" t="str">
-        <x:v>https://www.bikubenfonden.dk</x:v>
+        <x:v>https://duf.dk</x:v>
       </x:c>
       <x:c r="H12" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://duf.dk/tilskud-puljer/initiativstoetten/</x:v>
       </x:c>
       <x:c r="I12" t="str">
-        <x:v>Billedkunst; scenekunst; unge på kanten; sociale forandringer</x:v>
+        <x:v>Unge; demokratisk dannelse; demokratisk selvtillid; frivillighed; foreningsliv; klima og biodiversitet</x:v>
       </x:c>
       <x:c r="J12" t="str">
-        <x:v>Kunstnere; kulturinstitutioner; sociale organisationer; projekter efter opslag</x:v>
+        <x:v>Foreninger; projektgrupper; privatpersoner; frivilligdrevne initiativer</x:v>
       </x:c>
       <x:c r="K12" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Puljer med faste frister</x:v>
       </x:c>
       <x:c r="L12" t="str">
-        <x:v>Fokus på kunst og sociale indsatser.</x:v>
+        <x:v>Initiativstøtten er et kernematch for projekter af, for og med børn og unge.</x:v>
       </x:c>
       <x:c r="M12" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://duf.dk/tilskud-puljer/initiativstoetten/</x:v>
       </x:c>
       <x:c r="N12" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O12" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>tuborgfondet</x:v>
+        <x:v>oestifterne</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>Tuborgfondet</x:v>
+        <x:v>Østifterne</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
+        <x:v>Forening/fondslignende filantropisk aktør</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>To verify</x:v>
+        <x:v>Ikke relevant/forening</x:v>
       </x:c>
       <x:c r="E13" t="str">
         <x:v>Danmark</x:v>
       </x:c>
-      <x:c r="F13" t="str">
-        <x:v>København</x:v>
-      </x:c>
+      <x:c r="F13" t="str"/>
       <x:c r="G13" t="str">
-        <x:v>https://www.tuborgfondet.dk</x:v>
+        <x:v>https://www.oestifterne.dk</x:v>
       </x:c>
       <x:c r="H13" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://www.oestifterne.dk/uddelinger/uddelingspuljer/</x:v>
       </x:c>
       <x:c r="I13" t="str">
-        <x:v>Unge; fællesskaber; demokrati; grøn omstilling; civilsamfund</x:v>
+        <x:v>Lokale fællesskaber; deltagelse; trivsel; social forandring; skadeforebyggelse</x:v>
       </x:c>
       <x:c r="J13" t="str">
-        <x:v>Unge; foreninger; organisationer; lokale initiativer</x:v>
+        <x:v>Foreninger; organisationer; almennyttige initiativer</x:v>
       </x:c>
       <x:c r="K13" t="str">
         <x:v>Løbende og puljer</x:v>
       </x:c>
       <x:c r="L13" t="str">
-        <x:v>Fokus på unges engagement og handlekraft.</x:v>
+        <x:v>Relevant for fællesskab, deltagelse og social innovation; konkrete puljekriterier skal matche.</x:v>
       </x:c>
       <x:c r="M13" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://www.oestifterne.dk/uddelinger/uddelingspuljer/</x:v>
       </x:c>
       <x:c r="N13" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O13" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>egmont-fonden</x:v>
+        <x:v>lb-foreningen</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>Egmont Fonden</x:v>
+        <x:v>LB Foreningen</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>Erhvervsdrivende fond</x:v>
+        <x:v>Forening/fondslignende filantropisk aktør</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>Erhvervsstyrelsen</x:v>
+        <x:v>Ikke relevant/forening</x:v>
       </x:c>
       <x:c r="E14" t="str">
         <x:v>Danmark</x:v>
@@ -823,39 +869,39 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G14" t="str">
-        <x:v>https://www.egmontfonden.dk</x:v>
+        <x:v>https://www.lbforeningen.dk</x:v>
       </x:c>
       <x:c r="H14" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.lbforeningen.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="I14" t="str">
-        <x:v>Børn og unge; udsathed; læring; trivsel; social mobilitet</x:v>
+        <x:v>Fællesskaber; demokrati; bæredygtighed; socialt udsatte; frivillighed</x:v>
       </x:c>
       <x:c r="J14" t="str">
-        <x:v>Organisationer; institutioner; projekter efter opslag</x:v>
+        <x:v>Foreninger; organisationer; nationale regionale og lokale projekter</x:v>
       </x:c>
       <x:c r="K14" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Regionale og nationale uddelinger</x:v>
       </x:c>
       <x:c r="L14" t="str">
-        <x:v>Fokus på børn og unge i udsatte positioner.</x:v>
+        <x:v>Direkte match på demokrati, bæredygtighed og frivilligt funderede fællesskaber.</x:v>
       </x:c>
       <x:c r="M14" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.lbforeningen.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="N14" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O14" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>lauritzen-fonden</x:v>
+        <x:v>nordjyllandsfonden</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>Lauritzen Fonden</x:v>
+        <x:v>Nordjyllandsfonden</x:v>
       </x:c>
       <x:c r="C15" t="str">
         <x:v>Erhvervsdrivende fond</x:v>
@@ -867,189 +913,189 @@
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>Hellerup</x:v>
+        <x:v>Aalborg</x:v>
       </x:c>
       <x:c r="G15" t="str">
-        <x:v>https://lauritzenfonden.com</x:v>
+        <x:v>https://www.nordjyllandsfonden.dk</x:v>
       </x:c>
       <x:c r="H15" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://www.nordjyllandsfonden.dk/ansoeg</x:v>
       </x:c>
       <x:c r="I15" t="str">
-        <x:v>Udsatte børn og unge; maritimt; uddannelse; kultur; humanitære indsatser</x:v>
+        <x:v>Fællesskaber; kultur; fritid; sociale indsatser; børn og unge; frivillighed</x:v>
       </x:c>
       <x:c r="J15" t="str">
-        <x:v>Organisationer; institutioner; projekter</x:v>
+        <x:v>Foreninger; organisationer; lokale regionale og nationale projekter</x:v>
       </x:c>
       <x:c r="K15" t="str">
-        <x:v>Løbende og opslag</x:v>
+        <x:v>Løbende og uddelingsrunder</x:v>
       </x:c>
       <x:c r="L15" t="str">
-        <x:v>Har historisk maritime rødder og bred almennyttig uddeling.</x:v>
+        <x:v>Trods navnet støtter fonden projekter i hele Danmark; match er stærkest ved involverende fællesskaber.</x:v>
       </x:c>
       <x:c r="M15" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://www.nordjyllandsfonden.dk/ansoeg</x:v>
       </x:c>
       <x:c r="N15" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O15" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>william-demant-fonden</x:v>
+        <x:v>velliv-foreningen</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>William Demant Fonden</x:v>
+        <x:v>Velliv Foreningen</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Erhvervsdrivende fond</x:v>
+        <x:v>Forening/fondslignende filantropisk aktør</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Erhvervsstyrelsen</x:v>
+        <x:v>Ikke relevant/forening</x:v>
       </x:c>
       <x:c r="E16" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>Smørum</x:v>
+        <x:v>Ballerup</x:v>
       </x:c>
       <x:c r="G16" t="str">
-        <x:v>https://www.williamdemantfonden.dk</x:v>
+        <x:v>https://www.vellivforeningen.dk</x:v>
       </x:c>
       <x:c r="H16" t="str">
-        <x:v>https://www.williamdemantfonden.dk/ansoegning/</x:v>
+        <x:v>https://www.vellivforeningen.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="I16" t="str">
-        <x:v>Hørelse; sundhed; forskning; kultur; sociale formål</x:v>
+        <x:v>Mental sundhed; unge i overgangen til arbejdslivet; civilsamfund; fællesskaber; offentlig debat</x:v>
       </x:c>
       <x:c r="J16" t="str">
-        <x:v>Organisationer; institutioner; forskere; projekter</x:v>
+        <x:v>Civilsamfundsorganisationer; arbejdspladser; organisationer; forskere</x:v>
       </x:c>
       <x:c r="K16" t="str">
-        <x:v>Løbende og opslag</x:v>
+        <x:v>Løbende og puljer</x:v>
       </x:c>
       <x:c r="L16" t="str">
-        <x:v>Fokusområder bør valideres mod fondens aktuelle ansøgningsside.</x:v>
+        <x:v>Relevant for projekter om unges mentale sundhed og overgang til første job.</x:v>
       </x:c>
       <x:c r="M16" t="str">
-        <x:v>https://www.williamdemantfonden.dk/ansoegning/</x:v>
+        <x:v>https://www.vellivforeningen.dk/soeg-stoette</x:v>
       </x:c>
       <x:c r="N16" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O16" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>ole-kirks-fond</x:v>
+        <x:v>noerrebro-lokaludvalg</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>Ole Kirk's Fond</x:v>
+        <x:v>Nørrebro Lokaludvalg</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
+        <x:v>Kommunalt lokaludvalg</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>To verify</x:v>
+        <x:v>Københavns Kommune</x:v>
       </x:c>
       <x:c r="E17" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>Billund</x:v>
+        <x:v>København N</x:v>
       </x:c>
       <x:c r="G17" t="str">
-        <x:v>https://olekirksfond.dk</x:v>
+        <x:v>https://noerrebrolokaludvalg.kk.dk</x:v>
       </x:c>
       <x:c r="H17" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://noerrebrolokaludvalg.kk.dk/soeg-penge/</x:v>
       </x:c>
       <x:c r="I17" t="str">
-        <x:v>Børn; familier; trivsel; leg; læring; sociale indsatser</x:v>
+        <x:v>Lokaldemokrati; borgerinddragelse; netværk; sociale og kulturelle ressourcer; klima; social bæredygtighed</x:v>
       </x:c>
       <x:c r="J17" t="str">
-        <x:v>Organisationer; institutioner; projekter</x:v>
+        <x:v>Foreninger; projektgrupper; lokale aktører; borgere</x:v>
       </x:c>
       <x:c r="K17" t="str">
-        <x:v>Løbende og opslag</x:v>
+        <x:v>Faste runder og mindre pulje</x:v>
       </x:c>
       <x:c r="L17" t="str">
-        <x:v>Fokus på børns og familiers muligheder.</x:v>
+        <x:v>Projekter skal foregå på eller tydeligt gavne Nørrebro og helst have lokal forankring.</x:v>
       </x:c>
       <x:c r="M17" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://noerrebrolokaludvalg.kk.dk/soeg-penge/</x:v>
       </x:c>
       <x:c r="N17" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O17" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>kr-foundation</x:v>
+        <x:v>frederiksberg-kommune</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>KR Foundation</x:v>
+        <x:v>Frederiksberg Kommune</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
+        <x:v>Kommunal puljeaktør</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>To verify</x:v>
+        <x:v>Frederiksberg Kommune</x:v>
       </x:c>
       <x:c r="E18" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="F18" t="str">
-        <x:v>København</x:v>
+        <x:v>Frederiksberg</x:v>
       </x:c>
       <x:c r="G18" t="str">
-        <x:v>https://krfnd.org</x:v>
+        <x:v>https://www.frederiksberg.dk</x:v>
       </x:c>
       <x:c r="H18" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer</x:v>
       </x:c>
       <x:c r="I18" t="str">
-        <x:v>Klima; bæredygtighed; systemforandring; adfærd; policy</x:v>
+        <x:v>Kultur; fritid; fællesskaber; offentlige aktiviteter; børn og unge</x:v>
       </x:c>
       <x:c r="J18" t="str">
-        <x:v>Organisationer; NGO'er; internationale partnerskaber</x:v>
+        <x:v>Foreninger; organisationer; projektgrupper; borgere</x:v>
       </x:c>
       <x:c r="K18" t="str">
-        <x:v>Opslag/invitation</x:v>
+        <x:v>Løbende og faste runder</x:v>
       </x:c>
       <x:c r="L18" t="str">
-        <x:v>International klimafond med dansk base.</x:v>
+        <x:v>Projekter skal normalt finde sted på Frederiksberg og være offentligt tilgængelige eller målrettet relevante grupper.</x:v>
       </x:c>
       <x:c r="M18" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer</x:v>
       </x:c>
       <x:c r="N18" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O18" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>louis-hansen-fonden</x:v>
+        <x:v>koebenhavns-kommune</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>Louis-Hansen Fonden</x:v>
+        <x:v>Københavns Kommune</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
+        <x:v>Kommunal puljeaktør</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>To verify</x:v>
+        <x:v>Københavns Kommune</x:v>
       </x:c>
       <x:c r="E19" t="str">
         <x:v>Danmark</x:v>
@@ -1058,125 +1104,31 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G19" t="str">
-        <x:v>https://louishansenfonden.dk</x:v>
+        <x:v>https://www.kk.dk</x:v>
       </x:c>
       <x:c r="H19" t="str">
-        <x:v>https://louishansenfonden.dk/ansoegning/</x:v>
+        <x:v>https://www.kk.dk/brug-byen/kultur-og-projektstoette</x:v>
       </x:c>
       <x:c r="I19" t="str">
-        <x:v>Kunst; kultur; forskning; uddannelse; sociale formål</x:v>
+        <x:v>Unge; ungdomsdemokrati; foreningsudvikling; frivilligt socialt arbejde; kultur; mangfoldighed</x:v>
       </x:c>
       <x:c r="J19" t="str">
-        <x:v>Organisationer; institutioner; projekter</x:v>
+        <x:v>Foreninger; organisationer; unge; frivillige initiativer</x:v>
       </x:c>
       <x:c r="K19" t="str">
-        <x:v>Løbende og opslag</x:v>
+        <x:v>Løbende og faste runder</x:v>
       </x:c>
       <x:c r="L19" t="str">
-        <x:v>Støtteområder bør valideres mod fondens aktuelle ansøgningsside.</x:v>
+        <x:v>Kun programmer med direkte match til Sustainarys unge- og civilsamfundsarbejde er medtaget.</x:v>
       </x:c>
       <x:c r="M19" t="str">
-        <x:v>https://louishansenfonden.dk/ansoegning/</x:v>
+        <x:v>https://www.kk.dk/brug-byen/kultur-og-projektstoette</x:v>
       </x:c>
       <x:c r="N19" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="O19" t="str">
-        <x:v>to_verify</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" t="str">
-        <x:v>15-juni-fonden</x:v>
-      </x:c>
-      <x:c r="B20" t="str">
-        <x:v>15. Juni Fonden</x:v>
-      </x:c>
-      <x:c r="C20" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
-      </x:c>
-      <x:c r="D20" t="str">
-        <x:v>To verify</x:v>
-      </x:c>
-      <x:c r="E20" t="str">
-        <x:v>Danmark</x:v>
-      </x:c>
-      <x:c r="F20" t="str">
-        <x:v>København</x:v>
-      </x:c>
-      <x:c r="G20" t="str">
-        <x:v>https://www.15junifonden.dk</x:v>
-      </x:c>
-      <x:c r="H20" t="str">
-        <x:v>https://www.15junifonden.dk/ansoegning/</x:v>
-      </x:c>
-      <x:c r="I20" t="str">
-        <x:v>Natur; friluftsliv; kultur; sociale formål; humanitære formål</x:v>
-      </x:c>
-      <x:c r="J20" t="str">
-        <x:v>Organisationer; institutioner; projekter</x:v>
-      </x:c>
-      <x:c r="K20" t="str">
-        <x:v>Løbende og opslag</x:v>
-      </x:c>
-      <x:c r="L20" t="str">
-        <x:v>Støtteområder bør valideres mod fondens aktuelle ansøgningsside.</x:v>
-      </x:c>
-      <x:c r="M20" t="str">
-        <x:v>https://www.15junifonden.dk/ansoegning/</x:v>
-      </x:c>
-      <x:c r="N20" t="str">
-        <x:v>2026-06-08</x:v>
-      </x:c>
-      <x:c r="O20" t="str">
-        <x:v>to_verify</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" t="str">
-        <x:v>den-obelske-familiefond</x:v>
-      </x:c>
-      <x:c r="B21" t="str">
-        <x:v>Det Obelske Familiefond</x:v>
-      </x:c>
-      <x:c r="C21" t="str">
-        <x:v>Almennyttig fond/fondslignende</x:v>
-      </x:c>
-      <x:c r="D21" t="str">
-        <x:v>To verify</x:v>
-      </x:c>
-      <x:c r="E21" t="str">
-        <x:v>Danmark</x:v>
-      </x:c>
-      <x:c r="F21" t="str">
-        <x:v>Aalborg</x:v>
-      </x:c>
-      <x:c r="G21" t="str">
-        <x:v>https://obel.com</x:v>
-      </x:c>
-      <x:c r="H21" t="str">
-        <x:v>https://obel.com/ansoegning/</x:v>
-      </x:c>
-      <x:c r="I21" t="str">
-        <x:v>Kunst; kultur; sociale indsatser; uddannelse; civilsamfund</x:v>
-      </x:c>
-      <x:c r="J21" t="str">
-        <x:v>Organisationer; institutioner; projekter</x:v>
-      </x:c>
-      <x:c r="K21" t="str">
-        <x:v>Løbende og opslag</x:v>
-      </x:c>
-      <x:c r="L21" t="str">
-        <x:v>Nordjysk forankring bør valideres som geografisk kriterie ved konkrete ansøgninger.</x:v>
-      </x:c>
-      <x:c r="M21" t="str">
-        <x:v>https://obel.com/ansoegning/</x:v>
-      </x:c>
-      <x:c r="N21" t="str">
-        <x:v>2026-06-08</x:v>
-      </x:c>
-      <x:c r="O21" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1190,6 +1142,1836 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
+        <x:v>program_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>foundation_id</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>program_name</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>program_type</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>support_areas</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>applicant_types</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>geography</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>funding_use</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>amount_range</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>application_status</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>deadline_summary</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>application_url</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>source_url</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>last_checked</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
+        <x:v>verification_status</x:v>
+      </x:c>
+      <x:c r="P1" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>nordea-fonden-good-lives</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>nordea-fonden</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Støtte til gode liv</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>Projektstøtte</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Sundhed; motion; natur; kultur; fællesskaber; gode liv</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>Foreninger; organisationer; institutioner; lokale projekter</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Almennyttige projekter</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>Løbende og puljer</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>https://nordeafonden.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P2" t="str">
+        <x:v>Puljer og kriterier bør verificeres før brug.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>trygfonden-safety</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>trygfonden</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Tryghed og trivsel</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Projektstøtte</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Tryghed; sundhed; sikkerhed; trivsel; forskning; beredskab</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>Organisationer; institutioner; NGO'er; frivillige; forskere</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Projekter og forskning</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>Løbende og landsdækkende puljer</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>https://tryghed.dk/sog-stotte</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>https://tryghed.dk/sog-stotte</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P3" t="str">
+        <x:v>Støtter ikke privatpersoner eller kommercielle, politiske eller religiøse projekter.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>villum-research-calls</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>villum-fonden</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>VILLUM FONDEN opslag</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Call-baseret program</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Miljø og klima; børn unge og science; unge og uddannelse; kultur og samfund</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Forskere; institutioner; organisationer; projekter efter opslag</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Danmark og Europa</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Forskning uddannelse og almennyttige projekter</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Frister afhænger af konkrete calls</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P4" t="str">
+        <x:v>Prioritér kun opslag med tydeligt match til unge eller klima.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>velux-humanities-calls</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>velux-fonden</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>VELUX FONDEN opslag</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Call-baseret program</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Demokratisk bæredygtighed; sociale indsatser; human- og samfundsvidenskab; havmiljø</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Forskere; praktikere; institutioner; organisationer; projekter efter opslag</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Forskning praksis og almennyttige projekter</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>Frister afhænger af konkrete calls</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P5" t="str">
+        <x:v>Prioritér demokratisk bæredygtighed og sociale indsatser.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>bikuben-art-social</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>bikubenfonden</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Kunst og sociale forandringer</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Call-baseret program</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Billedkunst; scenekunst; unge på kanten; sociale forandringer</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Kunstnere; kulturinstitutioner; sociale organisationer; projekter efter opslag</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Kunstneriske og sociale projekter</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Opslag/calls</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P6" t="str">
+        <x:v>Fokus på kunst og sociale indsatser.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>tuborg-youth</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>tuborgfondet</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Unge og fællesskaber</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Projektstøtte</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Unge; fællesskaber; demokrati; grøn omstilling; civilsamfund</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Unge; foreninger; organisationer; lokale initiativer</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Projekter og initiativer</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="K7" t="str">
+        <x:v>Løbende og puljer</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P7" t="str">
+        <x:v>Fokus på unges engagement og handlekraft.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>egmont-children</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>egmont-fonden</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Børn og unge i udsatte positioner</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>Call-baseret program</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Børn og unge; udsathed; læring; trivsel; social mobilitet</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Organisationer; institutioner; projekter efter opslag</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Projekter og indsatser</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K8" t="str">
+        <x:v>Opslag/calls</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+      </x:c>
+      <x:c r="N8" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O8" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P8" t="str">
+        <x:v>Fokus på børn og unge i udsatte positioner.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>lauritzen-general</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>lauritzen-fonden</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Almennyttige uddelinger</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Projektstøtte</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Udsatte børn og unge; maritimt; uddannelse; kultur; humanitære indsatser</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Organisationer; institutioner; projekter</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Almennyttige projekter</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="K9" t="str">
+        <x:v>Løbende og opslag</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+      </x:c>
+      <x:c r="N9" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O9" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P9" t="str">
+        <x:v>Har historisk maritime rødder og bred almennyttig uddeling.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>ole-kirks-children</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>ole-kirks-fond</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Børn og familier</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Projektstøtte</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Børn; familier; trivsel; leg; læring; sociale indsatser</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Organisationer; institutioner; projekter</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Projekter for børn og familier</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="K10" t="str">
+        <x:v>Løbende og opslag</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+      </x:c>
+      <x:c r="N10" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O10" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P10" t="str">
+        <x:v>Fokus på børns og familiers muligheder.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>kr-climate</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>kr-foundation</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Climate funding</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>Invitation/opslag</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Klima; bæredygtighed; systemforandring; adfærd; policy</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Organisationer; NGO'er; internationale partnerskaber</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Internationalt</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Klimaindsatser</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>Efter invitation</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>Opslag/invitation</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+      </x:c>
+      <x:c r="N11" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="O11" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="P11" t="str">
+        <x:v>International klimafond med dansk base.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>duf-initiativstoetten</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>duf</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Initiativstøtten</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Pulje</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>Unge; demokratisk dannelse; demokratisk selvtillid; frivillighed; nyskabende projekter</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>Foreninger; projektgrupper; privatpersoner</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Frivilligdrevne projekter af for og med børn og unge</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>Op til 100.000 kr.; højere rammer for tematisk støtte</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K12" t="str">
+        <x:v>Næste frist 10. august 2026 kl. 12</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>https://duf.dk/tilskud-puljer/initiativstoetten/</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>https://duf.dk/tilskud-puljer/initiativstoetten/</x:v>
+      </x:c>
+      <x:c r="N12" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O12" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P12" t="str">
+        <x:v>Kernematch; unge skal deltage i planlægning udførelse og målgruppe.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>oestifterne-pools</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>oestifterne</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Uddelingspuljer</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Puljer</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>Lokale fællesskaber; deltagelse; trivsel; social forandring</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>Foreninger; organisationer; almennyttige initiativer</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>Østdanmark og efter konkret pulje</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Fællesskabs- og sociale indsatser</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>Efter pulje</x:v>
+      </x:c>
+      <x:c r="K13" t="str">
+        <x:v>Løbende og konkrete puljer</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>https://www.oestifterne.dk/uddelinger/uddelingspuljer/</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>https://www.oestifterne.dk/uddelinger/uddelingspuljer/</x:v>
+      </x:c>
+      <x:c r="N13" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O13" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P13" t="str">
+        <x:v>Vurder geografi og puljespecifikke kriterier før ansøgning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>lb-national-grants</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>lb-foreningen</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>Nationale og regionale uddelinger</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Uddelingsprogram</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>Fællesskaber; demokrati; bæredygtighed; socialt udsatte; frivillighed</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Foreninger; organisationer; regionale og nationale projekter</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Fællesskabsindsatser</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K14" t="str">
+        <x:v>Regionale og nationale uddelinger</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>https://www.lbforeningen.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>https://www.lbforeningen.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="N14" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O14" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P14" t="str">
+        <x:v>Stærkt tematisk match; kontrollér den aktuelle uddelings temaspor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>nordjyllandsfonden-community</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>nordjyllandsfonden</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>Fællesskaber</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Uddelingsprogram</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>Fællesskaber; sociale indsatser; børn og unge; kultur; fritid; frivillighed</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Foreninger; organisationer; lokale regionale og nationale projekter</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Involverende fællesskabsprojekter</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>Efter uddelingsrunde</x:v>
+      </x:c>
+      <x:c r="K15" t="str">
+        <x:v>Løbende og uddelingsrunder</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>https://www.nordjyllandsfonden.dk/ansoeg</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>https://www.nordjyllandsfonden.dk/ansoeg</x:v>
+      </x:c>
+      <x:c r="N15" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O15" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P15" t="str">
+        <x:v>Fonden støtter i hele Danmark og prioriterer involvering og social merværdi.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>velliv-youth-mental-health</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>velliv-foreningen</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>Unge og mental sundhed i arbejdslivet</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Pulje og projektstøtte</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>Unge; mental sundhed; overgang til første job; civilsamfund; offentlig debat</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Civilsamfundsorganisationer; arbejdspladser; organisationer</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Danmark</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Indsatser for mental sundhed og arbejdsliv</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>50.000-150.000 kr. i Fodfæste i fællesskab; større projekter varierer</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K16" t="str">
+        <x:v>Fodfæste i fællesskab: 26. august 2026; større ansøgninger løbende</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>https://www.vellivforeningen.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>https://www.vellivforeningen.dk/soeg-stoette</x:v>
+      </x:c>
+      <x:c r="N16" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O16" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P16" t="str">
+        <x:v>Relevant når projektet handler om unge i overgangen til arbejdslivet eller civilsamfundets støtte.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>noerrebro-byens-puls</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>noerrebro-lokaludvalg</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Byens Puls</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>Lokal pulje</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>Lokale aktiviteter; lokaldemokrati; fællesskab; netværk; borgerinddragelse</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>Foreninger; projektgrupper; lokale aktører; borgere</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Nørrebro</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Lokale aktiviteter og projekter</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>Op til 10.000 kr.</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K17" t="str">
+        <x:v>Næste frist 10. august 2026 ved midnat</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>https://noerrebrolokaludvalg.kk.dk/soeg-penge/</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>https://noerrebrolokaludvalg.kk.dk/byens-puls-er-aaben-igen-3/</x:v>
+      </x:c>
+      <x:c r="N17" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O17" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P17" t="str">
+        <x:v>Aktiviteter skal afholdes inden udgangen af 2026 og foregå på eller gavne Nørrebro.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>noerrebro-puljen</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>noerrebro-lokaludvalg</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>Nørrebro Puljen</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>Lokal pulje</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>Lokaldemokrati; borgerinddragelse; netværk; sociale og kulturelle ressourcer</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>Foreninger; projektgrupper; lokale aktører; borgere</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>Nørrebro</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Lokale projekter</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>Typisk 30.000-50.000 kr.; ingen formel øvre grænse</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="K18" t="str">
+        <x:v>To årlige ansøgningsrunder</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>https://noerrebrolokaludvalg.kk.dk/soeg-penge/</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>https://noerrebrolokaludvalg.kk.dk/soeg-penge/</x:v>
+      </x:c>
+      <x:c r="N18" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O18" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P18" t="str">
+        <x:v>Prioriterer dialogskabende og netværksdannende projekter samt demokratisk involvering.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>frederiksberg-hurtigpuljen</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>frederiksberg-kommune</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>Hurtigpuljen</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>Kommunal pulje</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>Kultur; fritid; offentlige aktiviteter; fællesskab</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Foreninger; organisationer; projektgrupper; borgere</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>Frederiksberg</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Mindre non-profit projekter</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>Op til 20.000 kr.</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K19" t="str">
+        <x:v>Løbende ansøgning; ingen behandling i juli</x:v>
+      </x:c>
+      <x:c r="L19" t="str">
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer/hurtigpuljen</x:v>
+      </x:c>
+      <x:c r="M19" t="str">
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer/hurtigpuljen</x:v>
+      </x:c>
+      <x:c r="N19" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O19" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P19" t="str">
+        <x:v>Projektet skal normalt finde sted på Frederiksberg og være offentligt tilgængeligt.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>frederiksberg-kultur-fritid</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>frederiksberg-kommune</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>Kultur- og fritidspuljen</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>Kommunal pulje</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>Kultur; fritid; offentlige aktiviteter; fællesskab</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>Foreninger; organisationer; projektgrupper</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Frederiksberg</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Større non-profit projekter</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>Op til 300.000 kr.</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K20" t="str">
+        <x:v>Frister 2. august og 15. september 2026</x:v>
+      </x:c>
+      <x:c r="L20" t="str">
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer/kultur-og-fritidspuljen</x:v>
+      </x:c>
+      <x:c r="M20" t="str">
+        <x:v>https://www.frederiksberg.dk/fritid-og-oplevelser/tilskud-fra-puljer/kultur-og-fritidspuljen</x:v>
+      </x:c>
+      <x:c r="N20" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O20" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P20" t="str">
+        <x:v>Relevant når Sustainary laver en offentlig kultur- eller fritidsaktivitet på Frederiksberg.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>kk-snabslanten</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>koebenhavns-kommune</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>Snabslanten</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>Kommunal ungdomspulje</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>Unge; ungdomsdemokrati; nyskabende kultur; frivillighed; offentlige arrangementer</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>Unge mellem 13 og 30 år bosat i Københavns Kommune</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>Københavns Kommune</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Små kultur- og ungdomsdemokratiske projekter</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>Samlet projektbudget under 30.000 kr.</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>Midlertidigt lukket</x:v>
+      </x:c>
+      <x:c r="K21" t="str">
+        <x:v>Åbner igen i august 2026; søg mindst 14 dage før projektet</x:v>
+      </x:c>
+      <x:c r="L21" t="str">
+        <x:v>https://snabslanten.kk.dk/retningslinjer</x:v>
+      </x:c>
+      <x:c r="M21" t="str">
+        <x:v>https://snabslanten.kk.dk/retningslinjer</x:v>
+      </x:c>
+      <x:c r="N21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O21" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P21" t="str">
+        <x:v>Ansøger skal være 13-30 år og bosat i København; egnet til ungedrevne Sustainary-initiativer.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>kk-udviklingspulje-boern-unge</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>koebenhavns-kommune</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>Udviklingspuljen for børn og unge</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Kommunal foreningspulje</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>Børn og unge under 25; foreningsudvikling; mangfoldighed; udsatte byområder</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>Godkendte folkeoplysende foreninger; initiativer der bliver folkeoplysende foreninger</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>Københavns Kommune</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Udviklingsprojekter for børn og unge</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>Op til 50.000 kr. uden medfinansiering; større projekter op til 75 procent</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>Åben</x:v>
+      </x:c>
+      <x:c r="K22" t="str">
+        <x:v>Løbende ansøgning</x:v>
+      </x:c>
+      <x:c r="L22" t="str">
+        <x:v>https://www.kk.dk/brug-byen/foreninger-og-fritidsliv/tilskud-og-puljer-for-foreninger-og-aftenskoler/soeg-udviklingspuljen-for-boern-og-unge</x:v>
+      </x:c>
+      <x:c r="M22" t="str">
+        <x:v>https://www.kk.dk/brug-byen/foreninger-og-fritidsliv/tilskud-og-puljer-for-foreninger-og-aftenskoler/soeg-udviklingspuljen-for-boern-og-unge</x:v>
+      </x:c>
+      <x:c r="N22" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O22" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P22" t="str">
+        <x:v>Sustainary skal være eller blive godkendt som folkeoplysende forening for at søge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>kk-paragraf-18</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>koebenhavns-kommune</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>§18-puljen</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Kommunal social pulje</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>Frivilligt socialt arbejde; udsatte børn og unge; netværk; rådgivning; frivillighed</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>Foreninger med frivilligt socialt arbejde</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Københavns Kommune</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>Sociale indsatser for københavnere</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>Varierer</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>Lukket</x:v>
+      </x:c>
+      <x:c r="K23" t="str">
+        <x:v>2027-runden lukkede 4. maj 2026; forventes årligt</x:v>
+      </x:c>
+      <x:c r="L23" t="str">
+        <x:v>https://www.kk.dk/brug-byen/kultur-og-projektstoette/stoette-til-socialt-arbejde/stoette-til-frivilligt-socialt-arbejde-ss18</x:v>
+      </x:c>
+      <x:c r="M23" t="str">
+        <x:v>https://www.kk.dk/brug-byen/kultur-og-projektstoette/stoette-til-socialt-arbejde/stoette-til-frivilligt-socialt-arbejde-ss18</x:v>
+      </x:c>
+      <x:c r="N23" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="O23" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+      <x:c r="P23" t="str">
+        <x:v>Kun relevant for projekter med frivilligt socialt arbejde og kommunens sociale målgrupper.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>deadline_id</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>program_id</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>deadline_type</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>opens_on</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>closes_on</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>recurrence</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>summary</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>last_checked</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
+        <x:v>verification_status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>nordea-fonden-good-lives-deadline</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>nordea-fonden-good-lives</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E2" t="str"/>
+      <x:c r="F2" t="str"/>
+      <x:c r="G2" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Løbende og puljer</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>trygfonden-safety-deadline</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>trygfonden-safety</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E3" t="str"/>
+      <x:c r="F3" t="str"/>
+      <x:c r="G3" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Løbende og landsdækkende puljer</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>villum-research-calls-deadline</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>villum-research-calls</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E4" t="str"/>
+      <x:c r="F4" t="str"/>
+      <x:c r="G4" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Frister afhænger af konkrete calls</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>velux-humanities-calls-deadline</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>velux-humanities-calls</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E5" t="str"/>
+      <x:c r="F5" t="str"/>
+      <x:c r="G5" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Frister afhænger af konkrete calls</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>bikuben-art-social-deadline</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>bikuben-art-social</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E6" t="str"/>
+      <x:c r="F6" t="str"/>
+      <x:c r="G6" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Opslag/calls</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>tuborg-youth-deadline</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>tuborg-youth</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E7" t="str"/>
+      <x:c r="F7" t="str"/>
+      <x:c r="G7" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Løbende og puljer</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>egmont-children-deadline</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>egmont-children</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E8" t="str"/>
+      <x:c r="F8" t="str"/>
+      <x:c r="G8" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Opslag/calls</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>lauritzen-general-deadline</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>lauritzen-general</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E9" t="str"/>
+      <x:c r="F9" t="str"/>
+      <x:c r="G9" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Løbende og opslag</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J9" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>ole-kirks-children-deadline</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>ole-kirks-children</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E10" t="str"/>
+      <x:c r="F10" t="str"/>
+      <x:c r="G10" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Løbende og opslag</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J10" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>kr-climate-deadline</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>kr-climate</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>invitation</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E11" t="str"/>
+      <x:c r="F11" t="str"/>
+      <x:c r="G11" t="str">
+        <x:v>Invitation/opslag</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Opslag/invitation</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>2026-06-08</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>duf-initiativstoetten-deadline</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>duf-initiativstoetten</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>fixed</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>upcoming</x:v>
+      </x:c>
+      <x:c r="E12" t="str"/>
+      <x:c r="F12" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>Flere årlige runder</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>Næste frist 10. august 2026 kl. 12</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J12" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>oestifterne-pools-deadline</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>oestifterne-pools</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E13" t="str"/>
+      <x:c r="F13" t="str"/>
+      <x:c r="G13" t="str">
+        <x:v>Efter pulje</x:v>
+      </x:c>
+      <x:c r="H13" t="str">
+        <x:v>Løbende og konkrete puljer</x:v>
+      </x:c>
+      <x:c r="I13" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J13" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>lb-national-grants-deadline</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>lb-national-grants</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E14" t="str"/>
+      <x:c r="F14" t="str"/>
+      <x:c r="G14" t="str">
+        <x:v>Efter opslag</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Regionale og nationale uddelinger</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J14" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>nordjyllandsfonden-community-deadline</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>nordjyllandsfonden-community</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E15" t="str"/>
+      <x:c r="F15" t="str"/>
+      <x:c r="G15" t="str">
+        <x:v>Efter uddelingsrunde</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Løbende og uddelingsrunder</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J15" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>velliv-youth-mental-health-deadline</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>velliv-youth-mental-health</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>fixed</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E16" t="str"/>
+      <x:c r="F16" t="str">
+        <x:v>2026-08-26</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Løbende og faste puljefrister</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Fodfæste i fællesskab har frist 26. august 2026; større ansøgninger løbende</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J16" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
+        <x:v>noerrebro-byens-puls-deadline</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>noerrebro-byens-puls</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>fixed</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E17" t="str"/>
+      <x:c r="F17" t="str">
+        <x:v>2026-08-10</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>Genåbnet pulje</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>Frist 10. august 2026 ved midnat</x:v>
+      </x:c>
+      <x:c r="I17" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
+        <x:v>noerrebro-puljen-deadline</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>noerrebro-puljen</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>call</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>to_verify</x:v>
+      </x:c>
+      <x:c r="E18" t="str"/>
+      <x:c r="F18" t="str"/>
+      <x:c r="G18" t="str">
+        <x:v>To årlige runder</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>Næste runde skal verificeres</x:v>
+      </x:c>
+      <x:c r="I18" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
+        <x:v>frederiksberg-hurtigpuljen-deadline</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>frederiksberg-hurtigpuljen</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E19" t="str"/>
+      <x:c r="F19" t="str"/>
+      <x:c r="G19" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>Løbende ansøgning; ingen behandling i juli</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
+        <x:v>frederiksberg-kultur-fritid-deadline</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>frederiksberg-kultur-fritid</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>fixed</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E20" t="str"/>
+      <x:c r="F20" t="str">
+        <x:v>2026-08-02</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>Fem årlige runder</x:v>
+      </x:c>
+      <x:c r="H20" t="str">
+        <x:v>Næste frist 2. august 2026; derefter 15. september</x:v>
+      </x:c>
+      <x:c r="I20" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" t="str">
+        <x:v>kk-snabslanten-deadline</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>kk-snabslanten</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>upcoming</x:v>
+      </x:c>
+      <x:c r="E21" t="str">
+        <x:v>2026-08-01</x:v>
+      </x:c>
+      <x:c r="F21" t="str"/>
+      <x:c r="G21" t="str">
+        <x:v>Løbende med sommerlukning</x:v>
+      </x:c>
+      <x:c r="H21" t="str">
+        <x:v>Åbner igen i august; minimum 14 dage før aktivitet</x:v>
+      </x:c>
+      <x:c r="I21" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J21" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" t="str">
+        <x:v>kk-udviklingspulje-boern-unge-deadline</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>kk-udviklingspulje-boern-unge</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>rolling</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>open</x:v>
+      </x:c>
+      <x:c r="E22" t="str"/>
+      <x:c r="F22" t="str"/>
+      <x:c r="G22" t="str">
+        <x:v>Løbende</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>Løbende ansøgning</x:v>
+      </x:c>
+      <x:c r="I22" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J22" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>kk-paragraf-18-deadline</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>kk-paragraf-18</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>annual</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>closed</x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>2026-01-01</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>2026-05-04</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>Årligt</x:v>
+      </x:c>
+      <x:c r="H23" t="str">
+        <x:v>2027-runden er lukket; overvåg næste årlige åbning</x:v>
+      </x:c>
+      <x:c r="I23" t="str">
+        <x:v>2026-07-02</x:v>
+      </x:c>
+      <x:c r="J23" t="str">
+        <x:v>source_checked</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
         <x:v>Dansk Fondsdatabase</x:v>
       </x:c>
       <x:c r="B1" t="str"/>
@@ -1205,24 +2987,24 @@
         <x:v>Fonde i seed</x:v>
       </x:c>
       <x:c r="B2" t="n">
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="D2" t="str">
         <x:v>København</x:v>
       </x:c>
       <x:c r="E2" t="n">
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Kilde-tjekket</x:v>
+        <x:v>Puljer i seed</x:v>
       </x:c>
       <x:c r="B3" t="n">
-        <x:v>6</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>Hellerup</x:v>
+        <x:v>Søborg</x:v>
       </x:c>
       <x:c r="E3" t="n">
         <x:v>2</x:v>
@@ -1230,24 +3012,24 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Skal verificeres</x:v>
+        <x:v>Løbende åbne puljer</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Søborg</x:v>
+        <x:v>Ballerup</x:v>
       </x:c>
       <x:c r="E4" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Seneste tjekdato</x:v>
-      </x:c>
-      <x:c r="B5" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>Puljer skal verificeres</x:v>
+      </x:c>
+      <x:c r="B5" t="n">
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Billund</x:v>
@@ -1258,13 +3040,13 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Primær datafil</x:v>
+        <x:v>Seneste tjekdato</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>data/fonde_seed.csv</x:v>
+        <x:v>2026-07-02</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Kgs. Lyngby</x:v>
+        <x:v>Frederiksberg</x:v>
       </x:c>
       <x:c r="E6" t="n">
         <x:v>1</x:v>
@@ -1272,13 +3054,13 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>SQLite-fil</x:v>
+        <x:v>Primær datafil</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>outputs/fonds_database.sqlite</x:v>
+        <x:v>data/fonde_seed.csv</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Smørum</x:v>
+        <x:v>Hellerup</x:v>
       </x:c>
       <x:c r="E7" t="n">
         <x:v>1</x:v>
@@ -1286,9 +3068,17 @@
     </x:row>
     <x:row r="8">
       <x:c r="D8" t="str">
-        <x:v>Aalborg</x:v>
+        <x:v>Kgs. Lyngby</x:v>
       </x:c>
       <x:c r="E8" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="D9" t="str">
+        <x:v>København N</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Modernize funding interface and links
</commit_message>
<xml_diff>
--- a/outputs/dansk_fonds_database.xlsx
+++ b/outputs/dansk_fonds_database.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonde" sheetId="1" r:id="R8ce1197ec5b543df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puljer" sheetId="2" r:id="R2bef05ec2eba43e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frister" sheetId="3" r:id="Rd794346f787f46f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opsummering" sheetId="4" r:id="R2412d0086b9947af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fonde" sheetId="1" r:id="Ra88fa1bba8c04a21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Puljer" sheetId="2" r:id="Ra6357745ed404034"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Frister" sheetId="3" r:id="Re903701f1eb942de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opsummering" sheetId="4" r:id="R456f89a1118a4921"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -401,10 +401,10 @@
         <x:v>Søborg</x:v>
       </x:c>
       <x:c r="G4" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+        <x:v>https://villumfonden.dk/da</x:v>
       </x:c>
       <x:c r="H4" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+        <x:v>https://villumfonden.dk/da/simpel-side/aktuelle-opslag-0</x:v>
       </x:c>
       <x:c r="I4" t="str">
         <x:v>Teknisk og naturvidenskabelig forskning; miljø og klima; børn unge og science; unge og uddannelse; kultur og samfund</x:v>
@@ -419,10 +419,10 @@
         <x:v>Relevant ved opslag om unge, uddannelse, miljø og klima.</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+        <x:v>https://villumfonden.dk/da/simpel-side/aktuelle-opslag-0</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O4" t="str">
         <x:v>source_checked</x:v>
@@ -448,10 +448,10 @@
         <x:v>Søborg</x:v>
       </x:c>
       <x:c r="G5" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+        <x:v>https://veluxfonden.dk/da</x:v>
       </x:c>
       <x:c r="H5" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+        <x:v>https://veluxfonden.dk/da/simpel-side/aktuelle-opslag</x:v>
       </x:c>
       <x:c r="I5" t="str">
         <x:v>Demokratisk bæredygtighed; sociale indsatser; human- og samfundsvidenskab; havmiljø</x:v>
@@ -463,13 +463,13 @@
         <x:v>Opslag/calls</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>Stærkt match ved opslag om demokratisk bæredygtighed og sociale indsatser.</x:v>
+        <x:v>Ansøgninger tager udgangspunkt i fondens aktuelle opslag.</x:v>
       </x:c>
       <x:c r="M5" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+        <x:v>https://veluxfonden.dk/da/artikel/saadan-soeger-du</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O5" t="str">
         <x:v>source_checked</x:v>
@@ -498,7 +498,7 @@
         <x:v>https://www.bikubenfonden.dk</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://www.bikubenfonden.dk/kom-i-dialog</x:v>
       </x:c>
       <x:c r="I6" t="str">
         <x:v>Billedkunst; scenekunst; unge på kanten; sociale forandringer</x:v>
@@ -507,19 +507,19 @@
         <x:v>Kunstnere; kulturinstitutioner; sociale organisationer; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Dialogbaseret</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>Fokus på kunst og sociale indsatser.</x:v>
+        <x:v>Bikubenfonden modtager ikke ansøgninger eller støtter enkeltstående indsatser; nye samarbejder starter med dialog.</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://www.bikubenfonden.dk/kom-i-dialog</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -542,10 +542,10 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G7" t="str">
-        <x:v>https://www.tuborgfondet.dk</x:v>
+        <x:v>https://tuborgfondet.dk</x:v>
       </x:c>
       <x:c r="H7" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://tuborgfondet.dk/projektstoette</x:v>
       </x:c>
       <x:c r="I7" t="str">
         <x:v>Unge; fællesskaber; demokrati; grøn omstilling; civilsamfund</x:v>
@@ -560,13 +560,13 @@
         <x:v>Fokus på unges engagement og handlekraft.</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://tuborgfondet.dk/projektstoette</x:v>
       </x:c>
       <x:c r="N7" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -589,10 +589,10 @@
         <x:v>København</x:v>
       </x:c>
       <x:c r="G8" t="str">
-        <x:v>https://www.egmontfonden.dk</x:v>
+        <x:v>https://www.egmont.dk</x:v>
       </x:c>
       <x:c r="H8" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.egmont.dk/saadan-ansoeger-i</x:v>
       </x:c>
       <x:c r="I8" t="str">
         <x:v>Børn og unge; udsathed; læring; trivsel; social mobilitet</x:v>
@@ -601,19 +601,19 @@
         <x:v>Organisationer; institutioner; projekter efter opslag</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Forespørgsel og invitation</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>Fokus på børn og unge i udsatte positioner.</x:v>
+        <x:v>En kort digital forespørgsel skal godkendes før en fuld ansøgning udarbejdes.</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.egmont.dk/saadan-ansoeger-i</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -639,7 +639,7 @@
         <x:v>https://lauritzenfonden.com</x:v>
       </x:c>
       <x:c r="H9" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://lauritzenfonden.com/soeg-stoette/</x:v>
       </x:c>
       <x:c r="I9" t="str">
         <x:v>Udsatte børn og unge; maritimt; uddannelse; kultur; humanitære indsatser</x:v>
@@ -654,13 +654,13 @@
         <x:v>Har historisk maritime rødder og bred almennyttig uddeling.</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://lauritzenfonden.com/soeg-stoette/</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -683,10 +683,10 @@
         <x:v>Billund</x:v>
       </x:c>
       <x:c r="G10" t="str">
-        <x:v>https://olekirksfond.dk</x:v>
+        <x:v>https://www.olekirksfond.dk</x:v>
       </x:c>
       <x:c r="H10" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://www.olekirksfond.dk/ansoegningsprocessen/</x:v>
       </x:c>
       <x:c r="I10" t="str">
         <x:v>Børn; familier; trivsel; leg; læring; sociale indsatser</x:v>
@@ -698,16 +698,16 @@
         <x:v>Løbende og opslag</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>Fokus på børns og familiers muligheder.</x:v>
+        <x:v>Ansøgninger indsendes via fondens digitale ansøgningsportal.</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://www.olekirksfond.dk/ansoegningsprocessen/</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -733,7 +733,7 @@
         <x:v>https://krfnd.org</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://krfnd.org/how-we-work/</x:v>
       </x:c>
       <x:c r="I11" t="str">
         <x:v>Klima; bæredygtighed; systemforandring; adfærd; policy</x:v>
@@ -742,19 +742,19 @@
         <x:v>Organisationer; NGO'er; internationale partnerskaber</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>Opslag/invitation</x:v>
+        <x:v>Kun invitation</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>International klimafond med dansk base.</x:v>
+        <x:v>KR Foundation modtager ikke uopfordrede ansøgninger; ansøgninger sker kun efter invitation.</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://krfnd.org/how-we-work/</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1325,13 +1325,13 @@
         <x:v>Frister afhænger af konkrete calls</x:v>
       </x:c>
       <x:c r="L4" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+        <x:v>https://villumfonden.dk/da/simpel-side/aktuelle-opslag-0</x:v>
       </x:c>
       <x:c r="M4" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/villum-fonden</x:v>
+        <x:v>https://villumfonden.dk/da/simpel-side/aktuelle-opslag-0</x:v>
       </x:c>
       <x:c r="N4" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O4" t="str">
         <x:v>source_checked</x:v>
@@ -1375,19 +1375,19 @@
         <x:v>Frister afhænger af konkrete calls</x:v>
       </x:c>
       <x:c r="L5" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+        <x:v>https://veluxfonden.dk/da/simpel-side/aktuelle-opslag</x:v>
       </x:c>
       <x:c r="M5" t="str">
-        <x:v>https://veluxfoundations.dk/da/group/foundation/velux-fonden</x:v>
+        <x:v>https://veluxfonden.dk/da/artikel/saadan-soeger-du</x:v>
       </x:c>
       <x:c r="N5" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O5" t="str">
         <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P5" t="str">
-        <x:v>Prioritér demokratisk bæredygtighed og sociale indsatser.</x:v>
+        <x:v>Ansøgninger tager udgangspunkt i et konkret aktuelt opslag.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1401,43 +1401,43 @@
         <x:v>Kunst og sociale forandringer</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Call-baseret program</x:v>
+        <x:v>Dialogbaseret samarbejde</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>Billedkunst; scenekunst; unge på kanten; sociale forandringer</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Kunstnere; kulturinstitutioner; sociale organisationer; projekter efter opslag</x:v>
+        <x:v>Kunstnere; kulturinstitutioner; sociale organisationer</x:v>
       </x:c>
       <x:c r="G6" t="str">
         <x:v>Danmark</x:v>
       </x:c>
       <x:c r="H6" t="str">
-        <x:v>Kunstneriske og sociale projekter</x:v>
+        <x:v>Kunstneriske og sociale samarbejder</x:v>
       </x:c>
       <x:c r="I6" t="str">
         <x:v>Varierer</x:v>
       </x:c>
       <x:c r="J6" t="str">
-        <x:v>Efter opslag</x:v>
+        <x:v>Dialogbaseret</x:v>
       </x:c>
       <x:c r="K6" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Ingen åbne ansøgninger</x:v>
       </x:c>
       <x:c r="L6" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://www.bikubenfonden.dk/kom-i-dialog</x:v>
       </x:c>
       <x:c r="M6" t="str">
-        <x:v>https://www.bikubenfonden.dk/soeg-stoette</x:v>
+        <x:v>https://www.bikubenfonden.dk/kom-i-dialog</x:v>
       </x:c>
       <x:c r="N6" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O6" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P6" t="str">
-        <x:v>Fokus på kunst og sociale indsatser.</x:v>
+        <x:v>Bikubenfonden modtager ikke ansøgninger eller støtter enkeltstående indsatser; nye samarbejder starter med dialog.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1475,19 +1475,19 @@
         <x:v>Løbende og puljer</x:v>
       </x:c>
       <x:c r="L7" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://tuborgfondet.dk/projektstoette</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>https://www.tuborgfondet.dk/soeg-stotte/</x:v>
+        <x:v>https://tuborgfondet.dk/projektstoette</x:v>
       </x:c>
       <x:c r="N7" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O7" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P7" t="str">
-        <x:v>Fokus på unges engagement og handlekraft.</x:v>
+        <x:v>Projektstøtte over 100.000 kr.; mindre initiativer kan høre under Drømmepuljen.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1501,13 +1501,13 @@
         <x:v>Børn og unge i udsatte positioner</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Call-baseret program</x:v>
+        <x:v>Forespørgselsbaseret program</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>Børn og unge; udsathed; læring; trivsel; social mobilitet</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>Organisationer; institutioner; projekter efter opslag</x:v>
+        <x:v>Organisationer; institutioner</x:v>
       </x:c>
       <x:c r="G8" t="str">
         <x:v>Danmark</x:v>
@@ -1519,25 +1519,25 @@
         <x:v>Varierer</x:v>
       </x:c>
       <x:c r="J8" t="str">
-        <x:v>Efter opslag</x:v>
+        <x:v>Forespørgsel</x:v>
       </x:c>
       <x:c r="K8" t="str">
-        <x:v>Opslag/calls</x:v>
+        <x:v>Forespørgsler behandles løbende</x:v>
       </x:c>
       <x:c r="L8" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.egmont.dk/saadan-ansoeger-i</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>https://www.egmontfonden.dk/ansoegning</x:v>
+        <x:v>https://www.egmont.dk/saadan-ansoeger-i</x:v>
       </x:c>
       <x:c r="N8" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O8" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P8" t="str">
-        <x:v>Fokus på børn og unge i udsatte positioner.</x:v>
+        <x:v>Send først en kort digital forespørgsel; fuld ansøgning udarbejdes kun efter invitation.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1575,16 +1575,16 @@
         <x:v>Løbende og opslag</x:v>
       </x:c>
       <x:c r="L9" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://lauritzenfonden.com/soeg-stoette/</x:v>
       </x:c>
       <x:c r="M9" t="str">
-        <x:v>https://lauritzenfonden.com/ansoegning/</x:v>
+        <x:v>https://lauritzenfonden.com/soeg-stoette/</x:v>
       </x:c>
       <x:c r="N9" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O9" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P9" t="str">
         <x:v>Har historisk maritime rødder og bred almennyttig uddeling.</x:v>
@@ -1625,19 +1625,19 @@
         <x:v>Løbende og opslag</x:v>
       </x:c>
       <x:c r="L10" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://www.olekirksfond.dk/ansoegningsprocessen/</x:v>
       </x:c>
       <x:c r="M10" t="str">
-        <x:v>https://olekirksfond.dk/ansoegning/</x:v>
+        <x:v>https://www.olekirksfond.dk/ansoegningsprocessen/</x:v>
       </x:c>
       <x:c r="N10" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O10" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P10" t="str">
-        <x:v>Fokus på børns og familiers muligheder.</x:v>
+        <x:v>Ansøgninger indsendes via fondens digitale GrantOne-portal.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1651,7 +1651,7 @@
         <x:v>Climate funding</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>Invitation/opslag</x:v>
+        <x:v>Invitation</x:v>
       </x:c>
       <x:c r="E11" t="str">
         <x:v>Klima; bæredygtighed; systemforandring; adfærd; policy</x:v>
@@ -1669,25 +1669,25 @@
         <x:v>Varierer</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>Efter invitation</x:v>
+        <x:v>Kun invitation</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>Opslag/invitation</x:v>
+        <x:v>Ingen uopfordrede ansøgninger</x:v>
       </x:c>
       <x:c r="L11" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://krfnd.org/how-we-work/</x:v>
       </x:c>
       <x:c r="M11" t="str">
-        <x:v>https://krfnd.org/apply-for-funding/</x:v>
+        <x:v>https://krfnd.org/how-we-work/</x:v>
       </x:c>
       <x:c r="N11" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="O11" t="str">
-        <x:v>to_verify</x:v>
+        <x:v>source_checked</x:v>
       </x:c>
       <x:c r="P11" t="str">
-        <x:v>International klimafond med dansk base.</x:v>
+        <x:v>KR Foundation modtager ikke uopfordrede ansøgninger; ansøgninger sker kun efter invitation.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -3029,7 +3029,7 @@
         <x:v>Puljer skal verificeres</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D5" t="str">
         <x:v>Billund</x:v>
@@ -3043,7 +3043,7 @@
         <x:v>Seneste tjekdato</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>2026-07-02</x:v>
+        <x:v>2026-07-26</x:v>
       </x:c>
       <x:c r="D6" t="str">
         <x:v>Frederiksberg</x:v>

</xml_diff>